<commit_message>
Aankoopdagboek per kwartaal: grootboekrekening, btw-code, status Yuki; tabblad in kwartaalpakket
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Samenvatting" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Verkopen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Aankopen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Btw-voorbereiding" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Bankafstemming" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Documenten" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Leningen" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="OSS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Samenvatting" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verkopen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aankopen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aankoopdagboek" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Btw-voorbereiding" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bankafstemming" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documenten" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leningen" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OSS" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Aankopen'!$A$3:$J$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Aankoopdagboek'!$A$3:$Q$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Voorbereid door het SmartPaw-financiënplatform op 2026-10-28. Voorbereiding: Pro-count controleert en dient in.</t>
+          <t>Voorbereid door het SmartPaw-financiënplatform op 2026-10-29. Voorbereiding: Pro-count controleert en dient in.</t>
         </is>
       </c>
     </row>
@@ -587,13 +589,13 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Tabbladen: Verkopen · Aankopen · Btw-voorbereiding · Bankafstemming · Documenten · Leningen · OSS</t>
+          <t>Tabbladen: Verkopen · Aankopen · Aankoopdagboek · Btw-voorbereiding · Bankafstemming · Documenten · Leningen · OSS</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1088,7 @@
         </is>
       </c>
       <c r="D23" s="10" t="n">
-        <v>8821.690000000001</v>
+        <v>9201.360000000001</v>
       </c>
     </row>
     <row r="24">
@@ -1490,7 +1492,7 @@
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Software &amp; abonnementen</t>
+          <t>Bankkosten</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -2481,6 +2483,2111 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Aankoopdagboek Q4 2026: 15 te boeken, 8 al in Yuki (ter controle), 1 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Factuurdatum</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Leverancier</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Btw-nr</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Factuurnr</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Rekening</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Rekeningnaam</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Btw-code</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Roosters</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>Maatstaf</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>Btw aftrekbaar</t>
+        </is>
+      </c>
+      <c r="L3" s="7" t="inlineStr">
+        <is>
+          <t>Verlegde btw</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Totaal betaald</t>
+        </is>
+      </c>
+      <c r="N3" s="7" t="inlineStr">
+        <is>
+          <t>Betaald op</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr">
+        <is>
+          <t>Betaald via</t>
+        </is>
+      </c>
+      <c r="P3" s="7" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="Q3" s="7" t="inlineStr">
+        <is>
+          <t>Opmerking</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>KBC Verzekeringen (polis 37630975, BA bedrijfspolis aansprakelijkheid)</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr"/>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>37630975</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>613210</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>GEEN</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>82</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="O4" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>KBC_BA-polis_37630975_2026-10-27.pdf</t>
+        </is>
+      </c>
+      <c r="Q4" s="8" t="inlineStr">
+        <is>
+          <t>geen btw / vrijgesteld</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr"/>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>33333736501041123</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>604000</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Aankopen van handelsgoederen</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>INVOER</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
+        </is>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>333</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9" t="n">
+        <v>69.93000000000001</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>333</v>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+        </is>
+      </c>
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>28560783836940336-28560783956940324</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="O6" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q6" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>28823801243971925-28794383930246982</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>517.01</v>
+      </c>
+      <c r="K7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="9" t="n">
+        <v>108.57</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>517.01</v>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q7" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>UAB Holo LT (Vilnius, LT)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>HOLO-202610-DB395</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>42.95</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>9.02</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>42.95</v>
+      </c>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="O8" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08_HoloAI_47.19USD.pdf</t>
+        </is>
+      </c>
+      <c r="Q8" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>Shopify International Ltd (IE)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>601792977</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>129.2</v>
+      </c>
+      <c r="K9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="9" t="n">
+        <v>27.13</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>129.2</v>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+        </is>
+      </c>
+      <c r="Q9" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Klaviyo Inc (Boston, US)</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>T9T7QHZO-0015</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>NEUDV</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59</t>
+        </is>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>63.59</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>63.59</v>
+      </c>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="O10" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10_Klaviyo_T9T7QHZO-0015_70USD.pdf</t>
+        </is>
+      </c>
+      <c r="Q10" s="8" t="inlineStr">
+        <is>
+          <t>dienst buiten EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>28770796055939105-28874006408951408</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>28719082304443821-28719082454443806</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O12" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q12" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>33333736501041123</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>604000</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Aankopen van handelsgoederen</t>
+        </is>
+      </c>
+      <c r="H13" s="8" t="inlineStr">
+        <is>
+          <t>INVOER</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
+        </is>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>779.1</v>
+      </c>
+      <c r="K13" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="9" t="n">
+        <v>163.61</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>779.1</v>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+        </is>
+      </c>
+      <c r="Q13" s="8" t="inlineStr">
+        <is>
+          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr"/>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>28824246560594057-28961227476895959</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="O14" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q14" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr"/>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>28937478365937539-29039294869089227</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H15" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="K15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="M15" s="9" t="n">
+        <v>800</v>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+        </is>
+      </c>
+      <c r="Q15" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>IE9692928F</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>28867302572955118-28867302652955110</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="G16" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="H16" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>621.34</v>
+      </c>
+      <c r="K16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="9" t="n">
+        <v>130.48</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>621.34</v>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="O16" s="8" t="inlineStr">
+        <is>
+          <t>434001 Mastercard Kaydee (2103)</t>
+        </is>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
+        </is>
+      </c>
+      <c r="Q16" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>bpost</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>12897185</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>611030</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>PORTKOSTEN</t>
+        </is>
+      </c>
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>8.470000000000001</v>
+      </c>
+      <c r="K17" s="9" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="L17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="9" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>bpost-bestelling 12897185 (26/10)</t>
+        </is>
+      </c>
+      <c r="Q17" s="8" t="inlineStr">
+        <is>
+          <t>Belgische btw 21%, aftrekbaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>te boeken</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Shenzhen Chongxin (Jess)</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr"/>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>PET2026102601</t>
+        </is>
+      </c>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>604000</t>
+        </is>
+      </c>
+      <c r="G18" s="8" t="inlineStr">
+        <is>
+          <t>Aankopen van handelsgoederen</t>
+        </is>
+      </c>
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>INVOER</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>4529.5</v>
+      </c>
+      <c r="K18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>951.1900000000001</v>
+      </c>
+      <c r="M18" s="9" t="n">
+        <v>4529.5</v>
+      </c>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27</t>
+        </is>
+      </c>
+      <c r="O18" s="8" t="inlineStr">
+        <is>
+          <t>550001 Revolut EUR</t>
+        </is>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+        </is>
+      </c>
+      <c r="Q18" s="8" t="inlineStr">
+        <is>
+          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>factuur ontbreekt</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>GODADDY*#7038004865</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr"/>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H19" s="8" t="inlineStr">
+        <is>
+          <t>NEUDV</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>167.76</v>
+      </c>
+      <c r="K19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>35.23</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>167.76</v>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr"/>
+      <c r="Q19" s="8" t="inlineStr">
+        <is>
+          <t>dienst buiten EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Yuki Works NV via Mollie</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr"/>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
+        </is>
+      </c>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>Belgische btw 21%, aftrekbaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr"/>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>616501</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME ZONDER MERK</t>
+        </is>
+      </c>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="K21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="9" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="M21" s="9" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+        </is>
+      </c>
+      <c r="Q21" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>METAPAY*MV4B</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr"/>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G22" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>EUDV</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>88 · 55 · 59</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="9" t="n">
+        <v>4.68</v>
+      </c>
+      <c r="M22" s="9" t="n">
+        <v>22.29</v>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr">
+        <is>
+          <t>434001 Mastercard Kaydee (2103)</t>
+        </is>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
+        </is>
+      </c>
+      <c r="Q22" s="8" t="inlineStr">
+        <is>
+          <t>dienst uit EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Pro-Count</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>615200</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
+          <t>Erelonen boekhouders en accountants</t>
+        </is>
+      </c>
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="K23" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="L23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="9" t="n">
+        <v>242</v>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
+        </is>
+      </c>
+      <c r="Q23" s="8" t="inlineStr">
+        <is>
+          <t>Belgische btw 21%, aftrekbaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>NEUDV</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>67.84</v>
+      </c>
+      <c r="K24" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>14.25</v>
+      </c>
+      <c r="M24" s="9" t="n">
+        <v>67.84</v>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O24" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
+        </is>
+      </c>
+      <c r="Q24" s="8" t="inlineStr">
+        <is>
+          <t>dienst buiten EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="F25" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="inlineStr">
+        <is>
+          <t>NEUDV</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="K25" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="9" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="M25" s="9" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
+        </is>
+      </c>
+      <c r="Q25" s="8" t="inlineStr">
+        <is>
+          <t>dienst buiten EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="F26" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="G26" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="inlineStr">
+        <is>
+          <t>NEUDV</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>87 · 56 · 59</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="K26" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="9" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="M26" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="O26" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P26" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
+        </is>
+      </c>
+      <c r="Q26" s="8" t="inlineStr">
+        <is>
+          <t>dienst buiten EU, btw verlegd</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr"/>
+      <c r="E27" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>611030</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
+          <t>PORTKOSTEN</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>BE21</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>82 · 59</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="K27" s="9" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="L27" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="9" t="n">
+        <v>6.78</v>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>550000 KBC zichtrekening</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Bpost (2026-10-21)</t>
+        </is>
+      </c>
+      <c r="Q27" s="8" t="inlineStr">
+        <is>
+          <t>Belgische btw 21%, aftrekbaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Totaal per grootboekrekening</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Rekening</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Naam</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Maatstaf</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Btw aftrekbaar</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>604000</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>Aankopen van handelsgoederen</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="9" t="n">
+        <v>5641.6</v>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>616502</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME MET MERK</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="D32" s="9" t="n">
+        <v>5138.35</v>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>611080</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>ABONNEMENTEN</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="D33" s="9" t="n">
+        <v>603.83</v>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>615200</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Erelonen boekhouders en accountants</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="9" t="n">
+        <v>200</v>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>616501</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>RECLAME ZONDER MERK</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="9" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>613210</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="9" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>611030</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>PORTKOSTEN</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D37" s="9" t="n">
+        <v>14.07</v>
+      </c>
+      <c r="E37" s="9" t="n">
+        <v>1.31</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:Q27"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2722,7 +4829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2804,16 +4911,16 @@
         <v>-331.19</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>9892.280000000001</v>
+        <v>10271.95</v>
       </c>
       <c r="E4" s="9" t="n">
         <v>-10585.81</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>-1024.72</v>
+        <v>-645.05</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="H4" s="10">
         <f>C4+D4+E4-F4</f>
@@ -2885,7 +4992,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Saldi teruggerekend vanaf de bankstand van 2026-10-28 (Ponto/Revolut). KBC-kredietkaart: zie Aankopen (rekening 'KBC-kaart'); afrekening via de zichtrekening.</t>
+          <t>Saldi teruggerekend vanaf de bankstand van 2026-10-29 (Ponto/Revolut). KBC-kredietkaart: zie Aankopen (rekening 'KBC-kaart'); afrekening via de zichtrekening.</t>
         </is>
       </c>
     </row>
@@ -2904,13 +5011,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -2924,7 +5031,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Bewijs per verrichting: 12 gekoppeld, 19 verklaard (geen factuur nodig, niet in deze lijst), 13 ontbreken. Facturen zitten in de map Facturen_Q4-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
+          <t>Bewijs per verrichting: 23 gekoppeld, 21 verklaard (geen factuur nodig, niet in deze lijst), 1 ontbreken. Facturen zitten in de map Facturen_Q4-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
         </is>
       </c>
     </row>
@@ -2963,20 +5070,20 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>GODADDY*#7038004865</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>-2.42</v>
+        <v>-167.76</v>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -2994,23 +5101,27 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-2.42</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -3020,11 +5131,11 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-22.29</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
@@ -3033,232 +5144,268 @@
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>-242</v>
+        <v>-22.29</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Company Pro plan fee</t>
+          <t>ALIBABA.COM</t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>-35</v>
+        <v>-333</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>KLAVIYO INC. SOFTWARE</t>
+          <t xml:space="preserve">FACEBK *QVA4B7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>-63.59</v>
+        <v>-800</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>GODADDY*#7038004865</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>-167.76</v>
+        <v>-242</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t xml:space="preserve">FACEBK *MYTGS7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>-67.84</v>
+        <v>-517.01</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>HOLO AI</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>-36.2</v>
+        <v>-42.95</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Holo AI HOLO-202610-DB395</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>SHOPIFY* 601792977</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>-72</v>
+        <v>-129.2</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+          <t>KLAVIYO INC. SOFTWARE</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>-6.78</v>
+        <v>-63.59</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Klaviyo T9T7QHZO-0015</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>FACEBK *CNGZB8S7A4</t>
+          <t xml:space="preserve">FACEBK *XX3GC6J8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>-621.34</v>
+        <v>-800</v>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
@@ -3267,54 +5414,62 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>KBC Verzekeringen</t>
+          <t>ALIBABA.COM</t>
         </is>
       </c>
       <c r="C16" s="9" t="n">
-        <v>-18.47</v>
+        <v>-779.1</v>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>ALIBABA.COM</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C17" s="9" t="n">
-        <v>-333</v>
+        <v>-67.84</v>
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -3324,19 +5479,19 @@
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *QVA4B7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t xml:space="preserve">FACEBK *J3XKX8W7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
@@ -3354,27 +5509,27 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *MYTGS7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>-517.01</v>
+        <v>-36.2</v>
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E19" s="8" t="inlineStr">
@@ -3384,23 +5539,23 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>HOLO AI</t>
+          <t xml:space="preserve">FACEBK *U6Y6G7J7A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>-42.95</v>
+        <v>-800</v>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
@@ -3414,27 +5569,27 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Holo AI HOLO-202610-DB395</t>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 601792977</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="C21" s="9" t="n">
-        <v>-129.2</v>
+        <v>-72</v>
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -3444,27 +5599,27 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *XX3GC6J8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>-800</v>
+        <v>-6.78</v>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -3474,27 +5629,27 @@
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>in Yuki: Bpost (2026-10-21)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>ALIBABA.COM</t>
+          <t xml:space="preserve">FACEBK *L8VFT7J8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C23" s="9" t="n">
-        <v>-779.1</v>
+        <v>-800</v>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -3504,23 +5659,23 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *J3XKX8W7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>FACEBK *CNGZB8S7A4</t>
         </is>
       </c>
       <c r="C24" s="9" t="n">
-        <v>-800</v>
+        <v>-621.34</v>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
@@ -3534,27 +5689,27 @@
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>Meta-factuur FBADS-210-106742402 (2026-10-23)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *U6Y6G7J7A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>bpost parcel</t>
         </is>
       </c>
       <c r="C25" s="9" t="n">
-        <v>-800</v>
+        <v>-8.6</v>
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -3564,27 +5719,27 @@
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>bpost-bestelling 12897185 (26/10)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *L8VFT7J8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>KBC Verzekeringen</t>
         </is>
       </c>
       <c r="C26" s="9" t="n">
-        <v>-800</v>
+        <v>-18.47</v>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -3594,27 +5749,27 @@
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>KBC vervaldagbericht polis 37630975 (2026-10-27 – 2026-11-26)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>bpost parcel</t>
+          <t>PET2026102601 30%</t>
         </is>
       </c>
       <c r="C27" s="9" t="n">
-        <v>-8.6</v>
+        <v>-4529.5</v>
       </c>
       <c r="D27" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NAKIJKEN</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -3623,36 +5778,6 @@
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>bpost-bestelling 12897185 (26/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-27</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>PET2026102601 30%</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="n">
-        <v>-4529.5</v>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>NAKIJKEN</t>
-        </is>
-      </c>
-      <c r="E28" s="8" t="inlineStr">
-        <is>
-          <t>gekoppeld</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Proforma PI-PET2026102601 (Shenzhen Chongxin, 27/10) – voorschot 30%</t>
         </is>
@@ -3663,7 +5788,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3820,7 +5945,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
GoDaddy-ontvangstbewijs 10/10 gekoppeld (Q4 compleet)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2513,7 +2513,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q4 2026: 15 te boeken, 8 al in Yuki (ter controle), 1 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q4 2026: 16 te boeken, 8 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -3137,70 +3137,74 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr"/>
+          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>EU MOSS EU372022543</t>
+        </is>
+      </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>28770796055939105-28874006408951408</t>
+          <t>7038004865</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>800</v>
+        <v>167.76</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>168</v>
+        <v>35.23</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>800</v>
+        <v>167.76</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>2026-10-10_GoDaddy_167.76.pdf</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>dienst buiten EU, btw verlegd</t>
         </is>
       </c>
     </row>
@@ -3212,7 +3216,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3223,7 +3227,7 @@
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>28719082304443821-28719082454443806</t>
+          <t>28770796055939105-28874006408951408</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -3260,7 +3264,7 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -3270,7 +3274,7 @@
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
@@ -3292,65 +3296,65 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>33333736501041123</t>
+          <t>28719082304443821-28719082454443806</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>779.1</v>
+        <v>800</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>163.61</v>
+        <v>168</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>779.1</v>
+        <v>800</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+          <t>dienst uit EU, btw verlegd</t>
         </is>
       </c>
     </row>
@@ -3362,70 +3366,70 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>28824246560594057-28961227476895959</t>
+          <t>33333736501041123</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>800</v>
+        <v>779.1</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>168</v>
+        <v>163.61</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>800</v>
+        <v>779.1</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
         </is>
       </c>
     </row>
@@ -3437,7 +3441,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3448,7 +3452,7 @@
       <c r="D15" s="8" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>28937478365937539-29039294869089227</t>
+          <t>28824246560594057-28961227476895959</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -3485,7 +3489,7 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
@@ -3495,7 +3499,7 @@
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
@@ -3512,7 +3516,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3520,14 +3524,10 @@
           <t>Meta Platforms Ireland</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>IE9692928F</t>
-        </is>
-      </c>
+      <c r="D16" s="8" t="inlineStr"/>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>28867302572955118-28867302652955110</t>
+          <t>28937478365937539-29039294869089227</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -3551,30 +3551,30 @@
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>621.34</v>
+        <v>800</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>130.48</v>
+        <v>168</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>621.34</v>
+        <v>800</v>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
@@ -3591,70 +3591,74 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr"/>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>IE9692928F</t>
+        </is>
+      </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>12897185</t>
+          <t>28867302572955118-28867302652955110</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>8.470000000000001</v>
+        <v>621.34</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0</v>
+        <v>130.48</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>8.6</v>
+        <v>621.34</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>bpost-bestelling 12897185 (26/10)</t>
+          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Belgische btw 21%, aftrekbaar</t>
+          <t>dienst uit EU, btw verlegd</t>
         </is>
       </c>
     </row>
@@ -3666,137 +3670,145 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin (Jess)</t>
+          <t>bpost</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>PET2026102601</t>
+          <t>12897185</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>4529.5</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>951.1900000000001</v>
+        <v>0</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>4529.5</v>
+        <v>8.6</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>550001 Revolut EUR</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+          <t>bpost-bestelling 12897185 (26/10)</t>
         </is>
       </c>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+          <t>Belgische btw 21%, aftrekbaar</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>factuur ontbreekt</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>GODADDY*#7038004865</t>
+          <t>Shenzhen Chongxin (Jess)</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
-      <c r="E19" s="8" t="inlineStr"/>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>PET2026102601</t>
+        </is>
+      </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
-        <v>167.76</v>
+        <v>4529.5</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>35.23</v>
+        <v>951.1900000000001</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>167.76</v>
+        <v>4529.5</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
-        </is>
-      </c>
-      <c r="P19" s="8" t="inlineStr"/>
+          <t>550001 Revolut EUR</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+        </is>
+      </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5043,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Bewijs per verrichting: 23 gekoppeld, 21 verklaard (geen factuur nodig, niet in deze lijst), 1 ontbreken. Facturen zitten in de map Facturen_Q4-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
+          <t>Bewijs per verrichting: 24 gekoppeld, 21 verklaard (geen factuur nodig, niet in deze lijst), 0 ontbreken. Facturen zitten in de map Facturen_Q4-2026 (bestandsnaam = datum_leverancier_bedrag).</t>
         </is>
       </c>
     </row>
@@ -5070,28 +5082,32 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>GODADDY*#7038004865</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>-167.76</v>
+        <v>-2.42</v>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>NONEU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>ontbreekt</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr"/>
+          <t>gekoppeld</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -5101,15 +5117,15 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>-2.42</v>
+        <v>-75.90000000000001</v>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -5119,7 +5135,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-10-02)</t>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
         </is>
       </c>
     </row>
@@ -5131,11 +5147,11 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>-75.90000000000001</v>
+        <v>-22.29</v>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
@@ -5149,27 +5165,27 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>ALIBABA.COM</t>
         </is>
       </c>
       <c r="C7" s="9" t="n">
-        <v>-22.29</v>
+        <v>-333</v>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -5179,27 +5195,27 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Mastercard (2026-10-02)</t>
+          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-03</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>ALIBABA.COM</t>
+          <t xml:space="preserve">FACEBK *QVA4B7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C8" s="9" t="n">
-        <v>-333</v>
+        <v>-800</v>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -5209,27 +5225,27 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Alibaba-ontvangstbewijs order 33333736501041123 (filters FF007 250 + FF009L 240)</t>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *QVA4B7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="C9" s="9" t="n">
-        <v>-800</v>
+        <v>-242</v>
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -5239,27 +5255,27 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t xml:space="preserve">FACEBK *MYTGS7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
         </is>
       </c>
       <c r="C10" s="9" t="n">
-        <v>-242</v>
+        <v>-517.01</v>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -5269,7 +5285,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-10-06)</t>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
         </is>
       </c>
     </row>
@@ -5281,11 +5297,11 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FACEBK *MYTGS7E8A4 IED04 X2K5 DUBLIN Betaling met </t>
+          <t>HOLO AI</t>
         </is>
       </c>
       <c r="C11" s="9" t="n">
-        <v>-517.01</v>
+        <v>-42.95</v>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
@@ -5299,23 +5315,23 @@
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>Holo AI HOLO-202610-DB395</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>HOLO AI</t>
+          <t>SHOPIFY* 601792977</t>
         </is>
       </c>
       <c r="C12" s="9" t="n">
-        <v>-42.95</v>
+        <v>-129.2</v>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
@@ -5329,27 +5345,27 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Holo AI HOLO-202610-DB395</t>
+          <t>Shopify-factuur 601792977 (mail 9/10)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>SHOPIFY* 601792977</t>
+          <t>KLAVIYO INC. SOFTWARE</t>
         </is>
       </c>
       <c r="C13" s="9" t="n">
-        <v>-129.2</v>
+        <v>-63.59</v>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>NONEU</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -5359,7 +5375,7 @@
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+          <t>Klaviyo T9T7QHZO-0015</t>
         </is>
       </c>
     </row>
@@ -5371,11 +5387,11 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>KLAVIYO INC. SOFTWARE</t>
+          <t>GODADDY*#7038004865</t>
         </is>
       </c>
       <c r="C14" s="9" t="n">
-        <v>-63.59</v>
+        <v>-167.76</v>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
@@ -5389,7 +5405,7 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo T9T7QHZO-0015</t>
+          <t>GoDaddy ontvangstbewijs 7038004865</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aankoopdagboek: voorschotten op proforma naar 406000 Vooruitbetalingen
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -2703,22 +2703,22 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J5" s="9" t="n">
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>69.93000000000001</v>
+        <v>0</v>
       </c>
       <c r="M5" s="9" t="n">
         <v>333</v>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+          <t>geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -3382,22 +3382,22 @@
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
@@ -3407,7 +3407,7 @@
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>163.61</v>
+        <v>0</v>
       </c>
       <c r="M14" s="9" t="n">
         <v>779.1</v>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+          <t>geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -3761,22 +3761,22 @@
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>INVOER</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59 (op invoeraangifte)</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
@@ -3786,7 +3786,7 @@
         <v>0</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>951.1900000000001</v>
+        <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
         <v>4529.5</v>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>goederen buiten EU, invoer-btw verlegd (art. 41) via invoeraangifte Widem</t>
+          <t>geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -4449,12 +4449,12 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>604000</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Aankopen van handelsgoederen</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="C31" s="8" t="n">

</xml_diff>

<commit_message>
Aankoopdagboek: btw-keuze in Yuki-termen (Shany 29/10); Yuki-betaling telt als geboekt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -2513,7 +2513,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q4 2026: 16 te boeken, 8 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q4 2026: 9 te boeken, 15 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="Q4" s="8" t="inlineStr">
         <is>
-          <t>geen btw / vrijgesteld</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>geen btw / vrijgesteld</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -2762,28 +2762,28 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>UAB Holo LT (Vilnius, LT)</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>28560783836940336-28560783956940324</t>
+          <t>HOLO-202610-DB395</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -2797,35 +2797,35 @@
         </is>
       </c>
       <c r="J6" s="9" t="n">
-        <v>800</v>
+        <v>42.95</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>168</v>
+        <v>9.02</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>800</v>
+        <v>42.95</v>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>2026-10-08_HoloAI_47.19USD.pdf</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -2837,28 +2837,28 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Shopify International Ltd (IE)</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>28823801243971925-28794383930246982</t>
+          <t>601792977</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -2872,35 +2872,35 @@
         </is>
       </c>
       <c r="J7" s="9" t="n">
-        <v>517.01</v>
+        <v>129.2</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>108.57</v>
+        <v>27.13</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>517.01</v>
+        <v>129.2</v>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>Shopify-factuur 601792977 (mail 9/10)</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -2912,18 +2912,18 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>UAB Holo LT (Vilnius, LT)</t>
+          <t>Klaviyo Inc (Boston, US)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>HOLO-202610-DB395</t>
+          <t>T9T7QHZO-0015</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -2938,29 +2938,29 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>42.95</v>
+        <v>63.59</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>9.02</v>
+        <v>13.35</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>42.95</v>
+        <v>63.59</v>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08_HoloAI_47.19USD.pdf</t>
+          <t>2026-10-10_Klaviyo_T9T7QHZO-0015_70USD.pdf</t>
         </is>
       </c>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -2987,18 +2987,22 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Shopify International Ltd (IE)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr"/>
+          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>EU MOSS EU372022543</t>
+        </is>
+      </c>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>601792977</t>
+          <t>7038004865</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -3013,29 +3017,29 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J9" s="9" t="n">
-        <v>129.2</v>
+        <v>167.76</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>27.13</v>
+        <v>35.23</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>129.2</v>
+        <v>167.76</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
@@ -3045,12 +3049,12 @@
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+          <t>2026-10-10_GoDaddy_167.76.pdf</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -3062,55 +3066,55 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo Inc (Boston, US)</t>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>T9T7QHZO-0015</t>
+          <t>33333736501041123</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>63.59</v>
+        <v>779.1</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>13.35</v>
+        <v>0</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>63.59</v>
+        <v>779.1</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
@@ -3120,12 +3124,12 @@
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10_Klaviyo_T9T7QHZO-0015_70USD.pdf</t>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
         </is>
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -3137,74 +3141,74 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>EU MOSS EU372022543</t>
+          <t>IE9692928F</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>7038004865</t>
+          <t>28867302572955118-28867302652955110</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>167.76</v>
+        <v>621.34</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>35.23</v>
+        <v>130.48</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>167.76</v>
+        <v>621.34</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10_GoDaddy_167.76.pdf</t>
+          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3216,130 +3220,130 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Shenzhen Chongxin (Jess)</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>28770796055939105-28874006408951408</t>
+          <t>PET2026102601</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>800</v>
+        <v>4529.5</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>800</v>
+        <v>4529.5</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>550001 Revolut EUR</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>28719082304443821-28719082454443806</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>800</v>
+        <v>2</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>800</v>
+        <v>2.42</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
@@ -3349,120 +3353,120 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>33333736501041123</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>779.1</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0</v>
+        <v>15.94</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>779.1</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>geen btw / vrijgesteld</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>28824246560594057-28961227476895959</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -3476,47 +3480,47 @@
         </is>
       </c>
       <c r="J15" s="9" t="n">
-        <v>800</v>
+        <v>22.29</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>168</v>
+        <v>4.68</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>800</v>
+        <v>22.29</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3527,7 +3531,7 @@
       <c r="D16" s="8" t="inlineStr"/>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>28937478365937539-29039294869089227</t>
+          <t>28560783836940336-28560783956940324</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -3564,7 +3568,7 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
@@ -3574,151 +3578,147 @@
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>IE9692928F</t>
-        </is>
-      </c>
+          <t>Pro-Count</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>28867302572955118-28867302652955110</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>621.34</v>
+        <v>200</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>130.48</v>
+        <v>0</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>621.34</v>
+        <v>242</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>12897185</t>
+          <t>28823801243971925-28794383930246982</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>8.470000000000001</v>
+        <v>517.01</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>0</v>
+        <v>108.57</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>8.6</v>
+        <v>517.01</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
@@ -3728,87 +3728,87 @@
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>bpost-bestelling 12897185 (26/10)</t>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Belgische btw 21%, aftrekbaar</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin (Jess)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>PET2026102601</t>
+          <t>28770796055939105-28874006408951408</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
-        <v>4529.5</v>
+        <v>800</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>4529.5</v>
+        <v>800</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>550001 Revolut EUR</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>geen btw / vrijgesteld</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3820,55 +3820,55 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>28719082304443821-28719082454443806</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J20" s="9" t="n">
-        <v>2</v>
+        <v>800</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>2.42</v>
+        <v>800</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
@@ -3878,12 +3878,12 @@
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-10-02)</t>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Belgische btw 21%, aftrekbaar</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3895,55 +3895,55 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr"/>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J21" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>67.84</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>15.94</v>
+        <v>14.25</v>
       </c>
       <c r="M21" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>67.84</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
@@ -3953,12 +3953,12 @@
       </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
         </is>
       </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -3970,18 +3970,18 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -3996,44 +3996,44 @@
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>22.29</v>
+        <v>36.2</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>4.68</v>
+        <v>7.6</v>
       </c>
       <c r="M22" s="9" t="n">
-        <v>22.29</v>
+        <v>36.2</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Mastercard (2026-10-02)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
         </is>
       </c>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>dienst uit EU, btw verlegd</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -4045,55 +4045,55 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>28824246560594057-28961227476895959</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J23" s="9" t="n">
-        <v>200</v>
+        <v>800</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="L23" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M23" s="9" t="n">
-        <v>242</v>
+        <v>800</v>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
@@ -4103,12 +4103,12 @@
       </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-10-06)</t>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>Belgische btw 21%, aftrekbaar</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -4131,7 +4131,7 @@
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -4155,20 +4155,20 @@
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>67.84</v>
+        <v>72</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>14.25</v>
+        <v>15.12</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>67.84</v>
+        <v>72</v>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
@@ -4178,12 +4178,12 @@
       </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
         </is>
       </c>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -4195,55 +4195,55 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J25" s="9" t="n">
-        <v>36.2</v>
+        <v>5.6</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>0</v>
+        <v>1.18</v>
       </c>
       <c r="L25" s="9" t="n">
-        <v>7.6</v>
+        <v>0</v>
       </c>
       <c r="M25" s="9" t="n">
-        <v>36.2</v>
+        <v>6.78</v>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="P25" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
+          <t>in Yuki: Bpost (2026-10-21)</t>
         </is>
       </c>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -4270,55 +4270,55 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>28937478365937539-29039294869089227</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>72</v>
+        <v>800</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="9" t="n">
-        <v>15.12</v>
+        <v>168</v>
       </c>
       <c r="M26" s="9" t="n">
-        <v>72</v>
+        <v>800</v>
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="P26" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>dienst buiten EU, btw verlegd</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -4345,18 +4345,18 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+          <t>bpost</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr"/>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>12897185</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -4380,20 +4380,20 @@
         </is>
       </c>
       <c r="J27" s="9" t="n">
-        <v>5.6</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>1.18</v>
+        <v>0.13</v>
       </c>
       <c r="L27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M27" s="9" t="n">
-        <v>6.78</v>
+        <v>8.6</v>
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
@@ -4403,12 +4403,12 @@
       </c>
       <c r="P27" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Bpost (2026-10-21)</t>
+          <t>bpost-bestelling 12897185 (26/10)</t>
         </is>
       </c>
       <c r="Q27" s="8" t="inlineStr">
         <is>
-          <t>Belgische btw 21%, aftrekbaar</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Betaling in Yuki telt enkel als geboekt voor facturen van vóór de ophaalperiode
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -2513,7 +2513,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q4 2026: 9 te boeken, 15 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q4 2026: 16 te boeken, 8 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -2762,28 +2762,28 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>UAB Holo LT (Vilnius, LT)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr"/>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>HOLO-202610-DB395</t>
+          <t>28560783836940336-28560783956940324</t>
         </is>
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
@@ -2797,30 +2797,30 @@
         </is>
       </c>
       <c r="J6" s="9" t="n">
-        <v>42.95</v>
+        <v>800</v>
       </c>
       <c r="K6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="9" t="n">
-        <v>9.02</v>
+        <v>168</v>
       </c>
       <c r="M6" s="9" t="n">
-        <v>42.95</v>
+        <v>800</v>
       </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="O6" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08_HoloAI_47.19USD.pdf</t>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
@@ -2837,28 +2837,28 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Shopify International Ltd (IE)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr"/>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>601792977</t>
+          <t>28823801243971925-28794383930246982</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H7" s="8" t="inlineStr">
@@ -2872,30 +2872,30 @@
         </is>
       </c>
       <c r="J7" s="9" t="n">
-        <v>129.2</v>
+        <v>517.01</v>
       </c>
       <c r="K7" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="9" t="n">
-        <v>27.13</v>
+        <v>108.57</v>
       </c>
       <c r="M7" s="9" t="n">
-        <v>129.2</v>
+        <v>517.01</v>
       </c>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O7" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Shopify-factuur 601792977 (mail 9/10)</t>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
@@ -2912,18 +2912,18 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Klaviyo Inc (Boston, US)</t>
+          <t>UAB Holo LT (Vilnius, LT)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>T9T7QHZO-0015</t>
+          <t>HOLO-202610-DB395</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -2938,29 +2938,29 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J8" s="9" t="n">
-        <v>63.59</v>
+        <v>42.95</v>
       </c>
       <c r="K8" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L8" s="9" t="n">
-        <v>13.35</v>
+        <v>9.02</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>63.59</v>
+        <v>42.95</v>
       </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="O8" s="8" t="inlineStr">
@@ -2970,12 +2970,12 @@
       </c>
       <c r="P8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10_Klaviyo_T9T7QHZO-0015_70USD.pdf</t>
+          <t>2026-10-08_HoloAI_47.19USD.pdf</t>
         </is>
       </c>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -2987,22 +2987,18 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>EU MOSS EU372022543</t>
-        </is>
-      </c>
+          <t>Shopify International Ltd (IE)</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr"/>
       <c r="E9" s="8" t="inlineStr">
         <is>
-          <t>7038004865</t>
+          <t>601792977</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -3017,29 +3013,29 @@
       </c>
       <c r="H9" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J9" s="9" t="n">
-        <v>167.76</v>
+        <v>129.2</v>
       </c>
       <c r="K9" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="9" t="n">
-        <v>35.23</v>
+        <v>27.13</v>
       </c>
       <c r="M9" s="9" t="n">
-        <v>167.76</v>
+        <v>129.2</v>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="O9" s="8" t="inlineStr">
@@ -3049,12 +3045,12 @@
       </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10_GoDaddy_167.76.pdf</t>
+          <t>Shopify-factuur 601792977 (mail 9/10)</t>
         </is>
       </c>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3066,55 +3062,55 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+          <t>Klaviyo Inc (Boston, US)</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr"/>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>33333736501041123</t>
+          <t>T9T7QHZO-0015</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J10" s="9" t="n">
-        <v>779.1</v>
+        <v>63.59</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>0</v>
+        <v>13.35</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>779.1</v>
+        <v>63.59</v>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O10" s="8" t="inlineStr">
@@ -3124,12 +3120,12 @@
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+          <t>2026-10-10_Klaviyo_T9T7QHZO-0015_70USD.pdf</t>
         </is>
       </c>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -3141,74 +3137,74 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>IE9692928F</t>
+          <t>EU MOSS EU372022543</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>28867302572955118-28867302652955110</t>
+          <t>7038004865</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>621.34</v>
+        <v>167.76</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>130.48</v>
+        <v>35.23</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>621.34</v>
+        <v>167.76</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
+          <t>2026-10-10_GoDaddy_167.76.pdf</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -3220,130 +3216,130 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin (Jess)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>PET2026102601</t>
+          <t>28770796055939105-28874006408951408</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J12" s="9" t="n">
-        <v>4529.5</v>
+        <v>800</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M12" s="9" t="n">
-        <v>4529.5</v>
+        <v>800</v>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
         <is>
-          <t>550001 Revolut EUR</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>28719082304443821-28719082454443806</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>2</v>
+        <v>800</v>
       </c>
       <c r="K13" s="9" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>2.42</v>
+        <v>800</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
@@ -3353,120 +3349,120 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-10-02)</t>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>33333736501041123</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>779.1</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>15.94</v>
+        <v>0</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>779.1</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>28824246560594057-28961227476895959</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
@@ -3480,30 +3476,30 @@
         </is>
       </c>
       <c r="J15" s="9" t="n">
-        <v>22.29</v>
+        <v>800</v>
       </c>
       <c r="K15" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="9" t="n">
-        <v>4.68</v>
+        <v>168</v>
       </c>
       <c r="M15" s="9" t="n">
-        <v>22.29</v>
+        <v>800</v>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Mastercard (2026-10-02)</t>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
@@ -3515,12 +3511,12 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3531,7 +3527,7 @@
       <c r="D16" s="8" t="inlineStr"/>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>28560783836940336-28560783956940324</t>
+          <t>28937478365937539-29039294869089227</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -3568,7 +3564,7 @@
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
@@ -3578,7 +3574,7 @@
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
@@ -3590,135 +3586,139 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr"/>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>IE9692928F</t>
+        </is>
+      </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>28867302572955118-28867302652955110</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>200</v>
+        <v>621.34</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>0</v>
+        <v>130.48</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>242</v>
+        <v>621.34</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Pro-Count (2026-10-06)</t>
+          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>bpost</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>28823801243971925-28794383930246982</t>
+          <t>12897185</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>517.01</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>108.57</v>
+        <v>0</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>517.01</v>
+        <v>8.6</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
@@ -3728,87 +3728,87 @@
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>bpost-bestelling 12897185 (26/10)</t>
         </is>
       </c>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>in Yuki</t>
+          <t>te boeken</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Shenzhen Chongxin (Jess)</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>28770796055939105-28874006408951408</t>
+          <t>PET2026102601</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
-        <v>800</v>
+        <v>4529.5</v>
       </c>
       <c r="K19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>800</v>
+        <v>4529.5</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>550001 Revolut EUR</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
         </is>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
@@ -3820,55 +3820,55 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>28719082304443821-28719082454443806</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J20" s="9" t="n">
-        <v>800</v>
+        <v>2</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>800</v>
+        <v>2.42</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O20" s="8" t="inlineStr">
@@ -3878,12 +3878,12 @@
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -3895,55 +3895,55 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr"/>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J21" s="9" t="n">
-        <v>67.84</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>14.25</v>
+        <v>15.94</v>
       </c>
       <c r="M21" s="9" t="n">
-        <v>67.84</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O21" s="8" t="inlineStr">
@@ -3953,12 +3953,12 @@
       </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
         </is>
       </c>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3970,18 +3970,18 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -3996,44 +3996,44 @@
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>36.2</v>
+        <v>22.29</v>
       </c>
       <c r="K22" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>7.6</v>
+        <v>4.68</v>
       </c>
       <c r="M22" s="9" t="n">
-        <v>36.2</v>
+        <v>22.29</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
         </is>
       </c>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -4045,55 +4045,55 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>28824246560594057-28961227476895959</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="H23" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J23" s="9" t="n">
-        <v>800</v>
+        <v>200</v>
       </c>
       <c r="K23" s="9" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="L23" s="9" t="n">
-        <v>168</v>
+        <v>0</v>
       </c>
       <c r="M23" s="9" t="n">
-        <v>800</v>
+        <v>242</v>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O23" s="8" t="inlineStr">
@@ -4103,12 +4103,12 @@
       </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
         </is>
       </c>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -4131,7 +4131,7 @@
       <c r="D24" s="8" t="inlineStr"/>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -4155,20 +4155,20 @@
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>72</v>
+        <v>67.84</v>
       </c>
       <c r="K24" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>15.12</v>
+        <v>14.25</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>72</v>
+        <v>67.84</v>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O24" s="8" t="inlineStr">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-16)</t>
         </is>
       </c>
       <c r="Q24" s="8" t="inlineStr">
@@ -4195,55 +4195,55 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D25" s="8" t="inlineStr"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H25" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J25" s="9" t="n">
-        <v>5.6</v>
+        <v>36.2</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>1.18</v>
+        <v>0</v>
       </c>
       <c r="L25" s="9" t="n">
-        <v>0</v>
+        <v>7.6</v>
       </c>
       <c r="M25" s="9" t="n">
-        <v>6.78</v>
+        <v>36.2</v>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O25" s="8" t="inlineStr">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="P25" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Bpost (2026-10-21)</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-15)</t>
         </is>
       </c>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -4270,55 +4270,55 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>HIGGSFIELD INC. US94105 SAN FRANCISCO Betaling met</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr"/>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>28937478365937539-29039294869089227</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G26" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J26" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="K26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="9" t="n">
-        <v>168</v>
+        <v>15.12</v>
       </c>
       <c r="M26" s="9" t="n">
-        <v>800</v>
+        <v>72</v>
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="O26" s="8" t="inlineStr">
@@ -4328,12 +4328,12 @@
       </c>
       <c r="P26" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>in Yuki: Higgsfield Inc (2026-10-20)</t>
         </is>
       </c>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -4345,18 +4345,18 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t>BPOST NV BE1000 BRUXELLES Betaling met KBC-Debetka</t>
         </is>
       </c>
       <c r="D27" s="8" t="inlineStr"/>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>12897185</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -4380,20 +4380,20 @@
         </is>
       </c>
       <c r="J27" s="9" t="n">
-        <v>8.470000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>0.13</v>
+        <v>1.18</v>
       </c>
       <c r="L27" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M27" s="9" t="n">
-        <v>8.6</v>
+        <v>6.78</v>
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="O27" s="8" t="inlineStr">
@@ -4403,7 +4403,7 @@
       </c>
       <c r="P27" s="8" t="inlineStr">
         <is>
-          <t>bpost-bestelling 12897185 (26/10)</t>
+          <t>in Yuki: Bpost (2026-10-21)</t>
         </is>
       </c>
       <c r="Q27" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Meta-kwitanties oktober als pdf gekoppeld
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -2820,7 +2820,7 @@
       </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-04_28560783836940336-28560783956940324.pdf</t>
         </is>
       </c>
       <c r="Q6" s="8" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="P7" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-08_28823801243971925-28794383930246982.pdf</t>
         </is>
       </c>
       <c r="Q7" s="8" t="inlineStr">
@@ -3274,7 +3274,7 @@
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-11_28770796055939105-28874006408951408.pdf</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
@@ -3349,7 +3349,7 @@
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-14_28719082304443821-28719082454443806.pdf</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
@@ -3499,7 +3499,7 @@
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-18_28824246560594057-28961227476895959.pdf</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>Meta_2026-10-21_28937478365937539-29039294869089227.pdf</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23_Meta_FBADS-210-106742402_621.34.pdf</t>
+          <t>Meta_2026-10-23_28867302572955118-28867302652955110.pdf</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28560783836940336-28560783956940324 (2026-10-04)</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5285,7 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28823801243971925-28794383930246982 (2026-10-08)</t>
         </is>
       </c>
     </row>
@@ -5435,7 +5435,7 @@
       </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28770796055939105-28874006408951408 (2026-10-11)</t>
         </is>
       </c>
     </row>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28719082304443821-28719082454443806 (2026-10-14)</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5585,7 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28824246560594057-28961227476895959 (2026-10-18)</t>
         </is>
       </c>
     </row>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21) – in Lucy/Yuki</t>
+          <t>Meta-kwitantie 28937478365937539-29039294869089227 (2026-10-21)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatisch doorsturen naar Yuki (nachtelijk) + leestest; Alibaba-filterorder op 604000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLjvFcZoD9WegLqrYozzyo
</commit_message>
<xml_diff>
--- a/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
+++ b/boekhouding/rapporten/SmartPaw_Q4-2026.xlsx
@@ -2488,7 +2488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q40"/>
+  <dimension ref="A1:Q41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2513,7 +2513,7 @@
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Aankoopdagboek Q4 2026: 16 te boeken, 10 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
+          <t>Aankoopdagboek Q4 2026: 15 te boeken, 11 al in Yuki (ter controle), 0 zonder factuur. Grootboekrekeningen volgens jullie rekeningschema; btw-codes: eigen code + roosters.</t>
         </is>
       </c>
     </row>
@@ -2703,22 +2703,22 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
         </is>
       </c>
       <c r="J5" s="9" t="n">
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="9" t="n">
-        <v>0</v>
+        <v>69.93000000000001</v>
       </c>
       <c r="M5" s="9" t="n">
         <v>333</v>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="Q5" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: invoer met verlegging (art. 41, invoeraangifte Widem)</t>
         </is>
       </c>
     </row>
@@ -3137,74 +3137,70 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>EU MOSS EU372022543</t>
-        </is>
-      </c>
+          <t>Meta Platforms Ireland</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr"/>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>7038004865</t>
+          <t>28770796055939105-28874006408951408</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>NEUDV</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
-          <t>87 · 56 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J11" s="9" t="n">
-        <v>167.76</v>
+        <v>800</v>
       </c>
       <c r="K11" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="9" t="n">
-        <v>35.23</v>
+        <v>168</v>
       </c>
       <c r="M11" s="9" t="n">
-        <v>167.76</v>
+        <v>800</v>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="O11" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-10_GoDaddy_167.76.pdf</t>
+          <t>Meta_2026-10-11_28770796055939105-28874006408951408.pdf</t>
         </is>
       </c>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Yuki: btw verlegd (dienst buiten EU)</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3212,7 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
@@ -3227,7 +3223,7 @@
       <c r="D12" s="8" t="inlineStr"/>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>28770796055939105-28874006408951408</t>
+          <t>28719082304443821-28719082454443806</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -3264,7 +3260,7 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="O12" s="8" t="inlineStr">
@@ -3274,7 +3270,7 @@
       </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
-          <t>Meta_2026-10-11_28770796055939105-28874006408951408.pdf</t>
+          <t>Meta_2026-10-14_28719082304443821-28719082454443806.pdf</t>
         </is>
       </c>
       <c r="Q12" s="8" t="inlineStr">
@@ -3296,65 +3292,65 @@
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
+          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr"/>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>28719082304443821-28719082454443806</t>
+          <t>33333736501041123</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>INVOER</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>87 · 56 · 59 (op invoeraangifte)</t>
         </is>
       </c>
       <c r="J13" s="9" t="n">
-        <v>800</v>
+        <v>779.1</v>
       </c>
       <c r="K13" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="9" t="n">
-        <v>168</v>
+        <v>163.61</v>
       </c>
       <c r="M13" s="9" t="n">
-        <v>800</v>
+        <v>779.1</v>
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="O13" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434000 Mastercard Henri (6682)</t>
         </is>
       </c>
       <c r="P13" s="8" t="inlineStr">
         <is>
-          <t>Meta_2026-10-14_28719082304443821-28719082454443806.pdf</t>
+          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
         </is>
       </c>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: invoer met verlegging (art. 41, invoeraangifte Widem)</t>
         </is>
       </c>
     </row>
@@ -3366,70 +3362,70 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin Technology Co. Ltd (via Alibaba.com Singapore)</t>
+          <t>Meta Platforms Ireland</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr"/>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>33333736501041123</t>
+          <t>28824246560594057-28961227476895959</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J14" s="9" t="n">
-        <v>779.1</v>
+        <v>800</v>
       </c>
       <c r="K14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="9" t="n">
-        <v>0</v>
+        <v>168</v>
       </c>
       <c r="M14" s="9" t="n">
-        <v>779.1</v>
+        <v>800</v>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="O14" s="8" t="inlineStr">
         <is>
-          <t>434000 Mastercard Henri (6682)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P14" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02_Alibaba_Shenzhen-Chongxin_1110.02.pdf</t>
+          <t>Meta_2026-10-18_28824246560594057-28961227476895959.pdf</t>
         </is>
       </c>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3441,7 +3437,7 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
@@ -3452,7 +3448,7 @@
       <c r="D15" s="8" t="inlineStr"/>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>28824246560594057-28961227476895959</t>
+          <t>28937478365937539-29039294869089227</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -3489,7 +3485,7 @@
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="O15" s="8" t="inlineStr">
@@ -3499,7 +3495,7 @@
       </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
-          <t>Meta_2026-10-18_28824246560594057-28961227476895959.pdf</t>
+          <t>Meta_2026-10-21_28937478365937539-29039294869089227.pdf</t>
         </is>
       </c>
       <c r="Q15" s="8" t="inlineStr">
@@ -3516,7 +3512,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -3524,10 +3520,14 @@
           <t>Meta Platforms Ireland</t>
         </is>
       </c>
-      <c r="D16" s="8" t="inlineStr"/>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>IE9692928F</t>
+        </is>
+      </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>28937478365937539-29039294869089227</t>
+          <t>28867302572955118-28867302652955110</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -3551,30 +3551,30 @@
         </is>
       </c>
       <c r="J16" s="9" t="n">
-        <v>800</v>
+        <v>621.34</v>
       </c>
       <c r="K16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>168</v>
+        <v>130.48</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>800</v>
+        <v>621.34</v>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="O16" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
-          <t>Meta_2026-10-21_28937478365937539-29039294869089227.pdf</t>
+          <t>Meta_2026-10-23_28867302572955118-28867302652955110.pdf</t>
         </is>
       </c>
       <c r="Q16" s="8" t="inlineStr">
@@ -3591,74 +3591,70 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Meta Platforms Ireland</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>IE9692928F</t>
-        </is>
-      </c>
+          <t>bpost</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr"/>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>28867302572955118-28867302652955110</t>
+          <t>12897185</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>611030</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>PORTKOSTEN</t>
         </is>
       </c>
       <c r="H17" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J17" s="9" t="n">
-        <v>621.34</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="K17" s="9" t="n">
-        <v>0</v>
+        <v>0.13</v>
       </c>
       <c r="L17" s="9" t="n">
-        <v>130.48</v>
+        <v>0</v>
       </c>
       <c r="M17" s="9" t="n">
-        <v>621.34</v>
+        <v>8.6</v>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="O17" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
-          <t>Meta_2026-10-23_28867302572955118-28867302652955110.pdf</t>
+          <t>bpost-bestelling 12897185 (26/10)</t>
         </is>
       </c>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -3670,145 +3666,145 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>bpost</t>
+          <t>Shenzhen Chongxin (Jess)</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr"/>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>12897185</t>
+          <t>PET2026102601</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
         <is>
-          <t>611030</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>PORTKOSTEN</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>GEEN</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>82</t>
         </is>
       </c>
       <c r="J18" s="9" t="n">
-        <v>8.470000000000001</v>
+        <v>4529.5</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="L18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>8.6</v>
+        <v>4529.5</v>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>550001 Revolut EUR</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
-          <t>bpost-bestelling 12897185 (26/10)</t>
+          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
         </is>
       </c>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: geen btw / vrijgesteld</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>te boeken</t>
+          <t>in Yuki</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Shenzhen Chongxin (Jess)</t>
+          <t>Yuki Works NV via Mollie</t>
         </is>
       </c>
       <c r="D19" s="8" t="inlineStr"/>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>PET2026102601</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H19" s="8" t="inlineStr">
         <is>
-          <t>GEEN</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I19" s="8" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J19" s="9" t="n">
-        <v>4529.5</v>
+        <v>2</v>
       </c>
       <c r="K19" s="9" t="n">
-        <v>0</v>
+        <v>0.42</v>
       </c>
       <c r="L19" s="9" t="n">
         <v>0</v>
       </c>
       <c r="M19" s="9" t="n">
-        <v>4529.5</v>
+        <v>2.42</v>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="O19" s="8" t="inlineStr">
         <is>
-          <t>550001 Revolut EUR</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P19" s="8" t="inlineStr">
         <is>
-          <t>2026-10-27_ShenzhenChongxin_PI-PET2026102601.pdf</t>
+          <t>in Yuki: Yuki works (2026-10-02)</t>
         </is>
       </c>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>Yuki: geen btw / vrijgesteld</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3821,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Yuki Works NV via Mollie</t>
+          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr"/>
@@ -3836,35 +3832,35 @@
       </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="G20" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>EUDV</t>
         </is>
       </c>
       <c r="I20" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>88 · 55 · 59</t>
         </is>
       </c>
       <c r="J20" s="9" t="n">
-        <v>2</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="K20" s="9" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="L20" s="9" t="n">
-        <v>0</v>
+        <v>15.94</v>
       </c>
       <c r="M20" s="9" t="n">
-        <v>2.42</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
@@ -3878,12 +3874,12 @@
       </c>
       <c r="P20" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Yuki works (2026-10-02)</t>
+          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
         </is>
       </c>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: intracommunautair diensten (verlegd)</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3896,7 @@
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>GOOGLE*WORKSPACE SMART IED02 R296 CC GOOGLE.COM Be</t>
+          <t>METAPAY*MV4B</t>
         </is>
       </c>
       <c r="D21" s="8" t="inlineStr"/>
@@ -3911,12 +3907,12 @@
       </c>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H21" s="8" t="inlineStr">
@@ -3930,16 +3926,16 @@
         </is>
       </c>
       <c r="J21" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>22.29</v>
       </c>
       <c r="K21" s="9" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="9" t="n">
-        <v>15.94</v>
+        <v>4.68</v>
       </c>
       <c r="M21" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>22.29</v>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
@@ -3948,12 +3944,12 @@
       </c>
       <c r="O21" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
+          <t>434001 Mastercard Kaydee (2103)</t>
         </is>
       </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Google Ireland Limited (2026-10-02)</t>
+          <t>in Yuki: Mastercard (2026-10-02)</t>
         </is>
       </c>
       <c r="Q21" s="8" t="inlineStr">
@@ -3970,70 +3966,70 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>METAPAY*MV4B</t>
+          <t>Pro-Count</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr"/>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="G22" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>EUDV</t>
+          <t>BE21</t>
         </is>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>88 · 55 · 59</t>
+          <t>82 · 59</t>
         </is>
       </c>
       <c r="J22" s="9" t="n">
-        <v>22.29</v>
+        <v>200</v>
       </c>
       <c r="K22" s="9" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="L22" s="9" t="n">
-        <v>4.68</v>
+        <v>0</v>
       </c>
       <c r="M22" s="9" t="n">
-        <v>22.29</v>
+        <v>242</v>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="O22" s="8" t="inlineStr">
         <is>
-          <t>434001 Mastercard Kaydee (2103)</t>
+          <t>550000 KBC zichtrekening</t>
         </is>
       </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
-          <t>in Yuki: Mastercard (2026-10-02)</t>
+          <t>in Yuki: Pro-Count (2026-10-06)</t>
         </is>
       </c>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>Yuki: intracommunautair diensten (verlegd)</t>
+          <t>Yuki: 21%</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4041,7 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
@@ -4056,7 +4052,7 @@
       <c r="D23" s="8" t="inlineStr"/>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>270345</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -4091,21 +4087,13 @@
       <c r="M23" s="9" t="n">
         <v>242</v>
       </c>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
+      <c r="N23" s="8" t="inlineStr"/>
       <c r="O23" s="8" t="inlineStr">
         <is>
-          <t>550000 KBC zichtrekening</t>
-        </is>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>in Yuki: Pro-Count (2026-10-06)</t>
-        </is>
-      </c>
+          <t xml:space="preserve"> nog te betalen (vervalt 2026-11-06)</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr"/>
       <c r="Q23" s="8" t="inlineStr">
         <is>
           <t>Yuki: 21%</t>
@@ -4120,62 +4108,74 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Pro-Count</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr"/>
+          <t>GoDaddy Europe Limited (Nottingham, UK)</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>EU MOSS EU372022543</t>
+        </is>
+      </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>270345</t>
+          <t>7038004865</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>BE21</t>
+          <t>NEUDV</t>
         </is>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>82 · 59</t>
+          <t>87 · 56 · 59</t>
         </is>
       </c>
       <c r="J24" s="9" t="n">
-        <v>200</v>
+        <v>167.76</v>
       </c>
       <c r="K24" s="9" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="L24" s="9" t="n">
-        <v>0</v>
+        <v>35.23</v>
       </c>
       <c r="M24" s="9" t="n">
-        <v>242</v>
-      </c>
-      <c r="N24" s="8" t="inlineStr"/>
+        <v>167.76</v>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
       <c r="O24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> nog te betalen (vervalt 2026-11-06)</t>
-        </is>
-      </c>
-      <c r="P24" s="8" t="inlineStr"/>
+          <t>434000 Mastercard Henri (6682)</t>
+        </is>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-10_GoDaddy_167.76.pdf</t>
+        </is>
+      </c>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>Yuki: 21%</t>
+          <t>Yuki: btw verlegd (dienst buiten EU)</t>
         </is>
       </c>
     </row>
@@ -4583,19 +4583,19 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>406000</t>
+          <t>616502</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>Vooruitbetalingen</t>
+          <t>RECLAME MET MERK</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D33" s="9" t="n">
-        <v>5641.6</v>
+        <v>5138.35</v>
       </c>
       <c r="E33" s="9" t="n">
         <v>0</v>
@@ -4604,19 +4604,19 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>616502</t>
+          <t>406000</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>RECLAME MET MERK</t>
+          <t>Vooruitbetalingen</t>
         </is>
       </c>
       <c r="C34" s="8" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D34" s="9" t="n">
-        <v>5138.35</v>
+        <v>4529.5</v>
       </c>
       <c r="E34" s="9" t="n">
         <v>0</v>
@@ -4625,82 +4625,82 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>611080</t>
+          <t>604000</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>ABONNEMENTEN</t>
+          <t>Aankopen van handelsgoederen</t>
         </is>
       </c>
       <c r="C35" s="8" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D35" s="9" t="n">
-        <v>603.83</v>
+        <v>1112.1</v>
       </c>
       <c r="E35" s="9" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>615200</t>
+          <t>611080</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Erelonen boekhouders en accountants</t>
+          <t>ABONNEMENTEN</t>
         </is>
       </c>
       <c r="C36" s="8" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>400</v>
+        <v>603.83</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>84</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>616651</t>
+          <t>615200</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
         <is>
-          <t>Beroepsbijdragen</t>
+          <t>Erelonen boekhouders en accountants</t>
         </is>
       </c>
       <c r="C37" s="8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D37" s="9" t="n">
-        <v>160</v>
+        <v>400</v>
       </c>
       <c r="E37" s="9" t="n">
-        <v>0</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>616501</t>
+          <t>616651</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>RECLAME ZONDER MERK</t>
+          <t>Beroepsbijdragen</t>
         </is>
       </c>
       <c r="C38" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>75.90000000000001</v>
+        <v>160</v>
       </c>
       <c r="E38" s="9" t="n">
         <v>0</v>
@@ -4709,19 +4709,19 @@
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>613210</t>
+          <t>616501</t>
         </is>
       </c>
       <c r="B39" s="8" t="inlineStr">
         <is>
-          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+          <t>RECLAME ZONDER MERK</t>
         </is>
       </c>
       <c r="C39" s="8" t="n">
         <v>1</v>
       </c>
       <c r="D39" s="9" t="n">
-        <v>18.47</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="E39" s="9" t="n">
         <v>0</v>
@@ -4730,21 +4730,42 @@
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
+          <t>613210</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>BURGERLIJKE AANSPRAKELIJKHEID</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" s="9" t="n">
+        <v>18.47</v>
+      </c>
+      <c r="E40" s="9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
           <t>611030</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B41" s="8" t="inlineStr">
         <is>
           <t>PORTKOSTEN</t>
         </is>
       </c>
-      <c r="C40" s="8" t="n">
+      <c r="C41" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D41" s="9" t="n">
         <v>14.07</v>
       </c>
-      <c r="E40" s="9" t="n">
+      <c r="E41" s="9" t="n">
         <v>1.31</v>
       </c>
     </row>

</xml_diff>